<commit_message>
New logistic cost model. Numerous bug fixes.
</commit_message>
<xml_diff>
--- a/inst/extdata/scenario_parameters.xlsx
+++ b/inst/extdata/scenario_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joe\pkgs\hpmicrosimr\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E4FF692-8EFF-4483-B2B1-A21357A53527}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B410D13-4209-4824-8DD1-C340A5015D71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="24" yWindow="744" windowWidth="23016" windowHeight="12216" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="282">
   <si>
     <t>category</t>
   </si>
@@ -516,9 +516,6 @@
     <t>not used, bias corrected at micro calibration stage</t>
   </si>
   <si>
-    <t>macro calibration: 3% may be consistent with RoI required by depositors</t>
-  </si>
-  <si>
     <t>scenario_BASE_1</t>
   </si>
   <si>
@@ -949,6 +946,48 @@
   </si>
   <si>
     <t>q_hotwater</t>
+  </si>
+  <si>
+    <t>ber_upgrade_marginal_cost_c0</t>
+  </si>
+  <si>
+    <t>low hanging fruit</t>
+  </si>
+  <si>
+    <t>inefficient house limit</t>
+  </si>
+  <si>
+    <t>rename to r.</t>
+  </si>
+  <si>
+    <t>present_bias_threshold</t>
+  </si>
+  <si>
+    <t>behaviour</t>
+  </si>
+  <si>
+    <t>present bias activation threshold</t>
+  </si>
+  <si>
+    <t>rebound activation threshold</t>
+  </si>
+  <si>
+    <t>rebound_threshold</t>
+  </si>
+  <si>
+    <t>no bias below this value but its probably heterogeneous</t>
+  </si>
+  <si>
+    <t>no rebound below this BER National Heat Study</t>
+  </si>
+  <si>
+    <t>labour cost share efficiency retrofit</t>
+  </si>
+  <si>
+    <t>guess</t>
+  </si>
+  <si>
+    <t>ber_upgrade_labour_cost_share</t>
   </si>
 </sst>
 </file>
@@ -1443,7 +1482,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="43.5" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.3">
@@ -1462,32 +1501,32 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>118</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="2" t="s">
         <v>126</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>128</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>129</v>
       </c>
       <c r="C5" s="2"/>
     </row>
@@ -1865,7 +1904,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C8E1679-ADB0-42D7-8103-5D0EB0C9F50E}">
-  <dimension ref="A1:F75"/>
+  <dimension ref="A1:F79"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -1898,135 +1937,135 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="B2" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="C2" s="9" t="s">
         <v>137</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>138</v>
       </c>
       <c r="D2" s="9">
         <v>2196</v>
       </c>
       <c r="E2" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="F2" t="s">
         <v>139</v>
-      </c>
-      <c r="F2" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D3" s="9">
         <v>16</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="B4" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="B4" s="13" t="s">
-        <v>135</v>
-      </c>
       <c r="C4" s="13" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D4" s="13">
         <v>30</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="B5" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="B5" s="12" t="s">
-        <v>135</v>
-      </c>
       <c r="C5" s="12" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D5" s="12">
         <v>40</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="B6" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="B6" s="13" t="s">
-        <v>135</v>
-      </c>
       <c r="C6" s="13" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D6" s="13">
         <v>60</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="B7" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="B7" s="13" t="s">
-        <v>135</v>
-      </c>
       <c r="C7" s="13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D7" s="13">
         <v>60</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="B8" s="14" t="s">
         <v>134</v>
       </c>
-      <c r="B8" s="14" t="s">
-        <v>135</v>
-      </c>
       <c r="C8" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D8" s="14">
         <v>60</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D9" s="10">
         <v>700</v>
@@ -2037,13 +2076,13 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D10" s="10">
         <v>0</v>
@@ -2052,13 +2091,13 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B11" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="C11" s="10" t="s">
         <v>143</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>144</v>
       </c>
       <c r="D11" s="10">
         <v>0</v>
@@ -2067,13 +2106,13 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="12" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D12" s="12">
         <v>150</v>
@@ -2084,13 +2123,13 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D13" s="13">
         <v>130</v>
@@ -2101,13 +2140,13 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D14" s="13">
         <v>200</v>
@@ -2118,13 +2157,13 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D15" s="13">
         <v>70</v>
@@ -2135,13 +2174,13 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="14" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D16" s="14">
         <v>120</v>
@@ -2152,79 +2191,82 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B17" s="13" t="s">
+        <v>217</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>216</v>
+      </c>
+      <c r="D17" s="13">
+        <v>110</v>
+      </c>
+      <c r="E17" s="14" t="s">
+        <v>219</v>
+      </c>
+      <c r="F17" t="s">
         <v>218</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>217</v>
-      </c>
-      <c r="D17" s="13">
-        <v>69.8</v>
-      </c>
-      <c r="E17" s="14" t="s">
-        <v>220</v>
-      </c>
-      <c r="F17" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B18" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="C18" s="13" t="s">
         <v>215</v>
       </c>
-      <c r="C18" s="13" t="s">
-        <v>216</v>
-      </c>
       <c r="D18" s="13">
-        <v>0.66700000000000004</v>
+        <v>0.81</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F18" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>149</v>
-      </c>
-      <c r="C19" s="11" t="s">
-        <v>254</v>
-      </c>
-      <c r="D19" s="11">
-        <v>2.25</v>
-      </c>
-      <c r="E19" s="11" t="s">
-        <v>203</v>
+      <c r="A19" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>270</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>268</v>
+      </c>
+      <c r="D19" s="13">
+        <v>0</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="F19" s="13" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="B20" s="11" t="s">
-        <v>149</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>253</v>
-      </c>
-      <c r="D20" s="11">
-        <v>2.75</v>
-      </c>
-      <c r="E20" s="11" t="s">
-        <v>203</v>
-      </c>
-      <c r="F20" t="s">
-        <v>250</v>
+      <c r="A20" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>279</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>281</v>
+      </c>
+      <c r="D20" s="13">
+        <v>0.3</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>202</v>
+      </c>
+      <c r="F20" s="13" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -2232,19 +2274,16 @@
         <v>18</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>244</v>
+        <v>148</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="D21" s="11">
-        <v>0.6</v>
+        <v>2.25</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>203</v>
-      </c>
-      <c r="F21" t="s">
-        <v>249</v>
+        <v>202</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
@@ -2252,19 +2291,19 @@
         <v>18</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>244</v>
+        <v>148</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="D22" s="11">
-        <v>0.85</v>
+        <v>2.75</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F22" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
@@ -2272,16 +2311,19 @@
         <v>18</v>
       </c>
       <c r="B23" s="11" t="s">
+        <v>243</v>
+      </c>
+      <c r="C23" s="11" t="s">
         <v>244</v>
       </c>
-      <c r="C23" s="11" t="s">
-        <v>247</v>
-      </c>
       <c r="D23" s="11">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>203</v>
+        <v>202</v>
+      </c>
+      <c r="F23" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -2289,78 +2331,81 @@
         <v>18</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>191</v>
+        <v>243</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="D24" s="11">
+        <v>0.85</v>
+      </c>
+      <c r="E24" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="F24" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>243</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>246</v>
+      </c>
+      <c r="D25" s="11">
+        <v>0.9</v>
+      </c>
+      <c r="E25" s="11" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>254</v>
+      </c>
+      <c r="D26" s="11">
         <v>0.75</v>
       </c>
-      <c r="E24" s="11" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="B25" s="15" t="s">
-        <v>190</v>
-      </c>
-      <c r="C25" s="15" t="s">
-        <v>256</v>
-      </c>
-      <c r="D25" s="15">
-        <v>1</v>
-      </c>
-      <c r="E25" s="15" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="15" t="s">
-        <v>161</v>
-      </c>
-      <c r="B26" s="15" t="s">
-        <v>150</v>
-      </c>
-      <c r="C26" s="15" t="s">
-        <v>151</v>
-      </c>
-      <c r="D26" s="15">
-        <v>17</v>
-      </c>
-      <c r="E26" s="15" t="s">
-        <v>9</v>
+      <c r="E26" s="11" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="15" t="s">
-        <v>161</v>
+        <v>18</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>152</v>
+        <v>189</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>153</v>
+        <v>255</v>
       </c>
       <c r="D27" s="15">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E27" s="15" t="s">
-        <v>9</v>
+        <v>202</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="D28" s="15">
         <v>17</v>
@@ -2371,13 +2416,13 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="D29" s="15">
         <v>12</v>
@@ -2388,16 +2433,16 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="B30" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="C30" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="B30" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="C30" s="15" t="s">
-        <v>192</v>
-      </c>
       <c r="D30" s="15">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="E30" s="15" t="s">
         <v>9</v>
@@ -2405,432 +2450,436 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>236</v>
+        <v>155</v>
       </c>
       <c r="C31" s="15" t="s">
-        <v>237</v>
+        <v>154</v>
       </c>
       <c r="D31" s="15">
-        <v>2.5</v>
-      </c>
-      <c r="E31" s="11" t="s">
-        <v>203</v>
+        <v>12</v>
+      </c>
+      <c r="E31" s="15" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B32" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="C32" s="15" t="s">
+        <v>191</v>
+      </c>
+      <c r="D32" s="15">
+        <v>25</v>
+      </c>
+      <c r="E32" s="15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>235</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>236</v>
+      </c>
+      <c r="D33" s="15">
+        <v>2.5</v>
+      </c>
+      <c r="E33" s="11" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A34" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="B34" s="15" t="s">
+        <v>238</v>
+      </c>
+      <c r="C34" s="15" t="s">
         <v>239</v>
       </c>
-      <c r="C32" s="15" t="s">
+      <c r="D34" s="15">
+        <v>2.5</v>
+      </c>
+      <c r="E34" s="11" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A35" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="B35" s="15" t="s">
+        <v>241</v>
+      </c>
+      <c r="C35" s="15" t="s">
+        <v>237</v>
+      </c>
+      <c r="D35" s="15">
+        <v>1.5</v>
+      </c>
+      <c r="E35" s="11" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="B36" s="15" t="s">
         <v>240</v>
       </c>
-      <c r="D32" s="15">
-        <v>2.5</v>
-      </c>
-      <c r="E32" s="11" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="15" t="s">
-        <v>161</v>
-      </c>
-      <c r="B33" s="15" t="s">
+      <c r="C36" s="15" t="s">
         <v>242</v>
       </c>
-      <c r="C33" s="15" t="s">
-        <v>238</v>
-      </c>
-      <c r="D33" s="15">
-        <v>1.5</v>
-      </c>
-      <c r="E33" s="11" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="15" t="s">
-        <v>161</v>
-      </c>
-      <c r="B34" s="15" t="s">
-        <v>241</v>
-      </c>
-      <c r="C34" s="15" t="s">
-        <v>243</v>
-      </c>
-      <c r="D34" s="15">
+      <c r="D36" s="15">
         <v>3</v>
       </c>
-      <c r="E34" s="11" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="21" t="s">
-        <v>161</v>
-      </c>
-      <c r="B35" s="21" t="s">
-        <v>252</v>
-      </c>
-      <c r="C35" s="21" t="s">
+      <c r="E36" s="11" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" s="21" t="s">
+        <v>160</v>
+      </c>
+      <c r="B37" s="21" t="s">
         <v>251</v>
       </c>
-      <c r="D35" s="21">
+      <c r="C37" s="21" t="s">
+        <v>250</v>
+      </c>
+      <c r="D37" s="21">
         <v>2</v>
       </c>
-      <c r="E35" s="21" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="21" t="s">
-        <v>18</v>
-      </c>
-      <c r="B36" s="21" t="s">
-        <v>260</v>
-      </c>
-      <c r="C36" s="21" t="s">
-        <v>261</v>
-      </c>
-      <c r="D36" s="21">
-        <v>15</v>
-      </c>
-      <c r="E36" s="21" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="21" t="s">
-        <v>18</v>
-      </c>
-      <c r="B37" s="21" t="s">
-        <v>263</v>
-      </c>
-      <c r="C37" s="21" t="s">
-        <v>268</v>
-      </c>
-      <c r="D37" s="21">
-        <v>30</v>
-      </c>
       <c r="E37" s="21" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="21" t="s">
         <v>18</v>
       </c>
       <c r="B38" s="21" t="s">
+        <v>259</v>
+      </c>
+      <c r="C38" s="21" t="s">
+        <v>260</v>
+      </c>
+      <c r="D38" s="21">
+        <v>15</v>
+      </c>
+      <c r="E38" s="21" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="B39" s="21" t="s">
+        <v>262</v>
+      </c>
+      <c r="C39" s="21" t="s">
+        <v>267</v>
+      </c>
+      <c r="D39" s="21">
+        <v>30</v>
+      </c>
+      <c r="E39" s="21" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="B40" s="21" t="s">
+        <v>263</v>
+      </c>
+      <c r="C40" s="21" t="s">
         <v>264</v>
       </c>
-      <c r="C38" s="21" t="s">
-        <v>265</v>
-      </c>
-      <c r="D38" s="21">
+      <c r="D40" s="21">
         <v>8</v>
       </c>
-      <c r="E38" s="21" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="16" t="s">
+      <c r="E40" s="21" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="B39" s="16" t="s">
+      <c r="B41" s="16" t="s">
+        <v>256</v>
+      </c>
+      <c r="C41" s="16" t="s">
         <v>257</v>
       </c>
-      <c r="C39" s="16" t="s">
-        <v>258</v>
-      </c>
-      <c r="D39" s="16">
+      <c r="D41" s="16">
         <v>0.75</v>
       </c>
-      <c r="E39" s="16"/>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="11" t="s">
-        <v>167</v>
-      </c>
-      <c r="B40" s="11" t="s">
-        <v>204</v>
-      </c>
-      <c r="C40" s="11" t="s">
-        <v>169</v>
-      </c>
-      <c r="D40" s="11">
-        <v>11.8</v>
-      </c>
-      <c r="E40" s="11"/>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="11" t="s">
-        <v>167</v>
-      </c>
-      <c r="B41" s="11" t="s">
+      <c r="E41" s="16"/>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="B42" s="11" t="s">
+        <v>203</v>
+      </c>
+      <c r="C42" s="11" t="s">
         <v>168</v>
-      </c>
-      <c r="C41" s="11" t="s">
-        <v>170</v>
-      </c>
-      <c r="D41" s="11">
-        <v>11.8</v>
-      </c>
-      <c r="E41" s="11"/>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="11" t="s">
-        <v>167</v>
-      </c>
-      <c r="B42" s="11" t="s">
-        <v>168</v>
-      </c>
-      <c r="C42" s="11" t="s">
-        <v>171</v>
       </c>
       <c r="D42" s="11">
         <v>11.8</v>
       </c>
       <c r="E42" s="11"/>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="B43" s="11" t="s">
         <v>167</v>
       </c>
-      <c r="B43" s="11" t="s">
-        <v>168</v>
-      </c>
       <c r="C43" s="11" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="D43" s="11">
         <v>11.8</v>
       </c>
       <c r="E43" s="11"/>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="B44" s="11" t="s">
         <v>167</v>
       </c>
-      <c r="B44" s="11" t="s">
+      <c r="C44" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="D44" s="11">
+        <v>11.8</v>
+      </c>
+      <c r="E44" s="11"/>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="B45" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="C45" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="D45" s="11">
+        <v>11.8</v>
+      </c>
+      <c r="E45" s="11"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="B46" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="C46" s="11" t="s">
         <v>173</v>
-      </c>
-      <c r="C44" s="11" t="s">
-        <v>174</v>
-      </c>
-      <c r="D44" s="11">
-        <v>13.2</v>
-      </c>
-      <c r="E44" s="11"/>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A45" s="11" t="s">
-        <v>167</v>
-      </c>
-      <c r="B45" s="11" t="s">
-        <v>173</v>
-      </c>
-      <c r="C45" s="11" t="s">
-        <v>175</v>
-      </c>
-      <c r="D45" s="11">
-        <v>13.2</v>
-      </c>
-      <c r="E45" s="11"/>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46" s="11" t="s">
-        <v>167</v>
-      </c>
-      <c r="B46" s="11" t="s">
-        <v>173</v>
-      </c>
-      <c r="C46" s="11" t="s">
-        <v>176</v>
       </c>
       <c r="D46" s="11">
         <v>13.2</v>
       </c>
       <c r="E46" s="11"/>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B47" s="11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C47" s="11" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="D47" s="11">
         <v>13.2</v>
       </c>
       <c r="E47" s="11"/>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B48" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="C48" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="D48" s="11">
+        <v>13.2</v>
+      </c>
+      <c r="E48" s="11"/>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A49" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="B49" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="C49" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="D49" s="11">
+        <v>13.2</v>
+      </c>
+      <c r="E49" s="11"/>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A50" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="B50" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="C50" s="11" t="s">
         <v>178</v>
-      </c>
-      <c r="C48" s="11" t="s">
-        <v>179</v>
-      </c>
-      <c r="D48" s="11">
-        <v>35.4</v>
-      </c>
-      <c r="E48" s="11"/>
-      <c r="F48" s="11"/>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A49" s="11" t="s">
-        <v>167</v>
-      </c>
-      <c r="B49" s="11" t="s">
-        <v>178</v>
-      </c>
-      <c r="C49" s="11" t="s">
-        <v>180</v>
-      </c>
-      <c r="D49" s="11">
-        <v>35.4</v>
-      </c>
-      <c r="E49" s="11"/>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A50" s="11" t="s">
-        <v>167</v>
-      </c>
-      <c r="B50" s="11" t="s">
-        <v>178</v>
-      </c>
-      <c r="C50" s="11" t="s">
-        <v>181</v>
       </c>
       <c r="D50" s="11">
         <v>35.4</v>
       </c>
       <c r="E50" s="11"/>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F50" s="11"/>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B51" s="11" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C51" s="11" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D51" s="11">
         <v>35.4</v>
       </c>
       <c r="E51" s="11"/>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B52" s="11" t="s">
-        <v>227</v>
+        <v>177</v>
       </c>
       <c r="C52" s="11" t="s">
-        <v>230</v>
+        <v>180</v>
       </c>
       <c r="D52" s="11">
-        <v>0.4</v>
+        <v>35.4</v>
       </c>
       <c r="E52" s="11"/>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B53" s="11" t="s">
-        <v>227</v>
+        <v>177</v>
       </c>
       <c r="C53" s="11" t="s">
-        <v>231</v>
+        <v>181</v>
       </c>
       <c r="D53" s="11">
-        <v>0.4</v>
+        <v>35.4</v>
       </c>
       <c r="E53" s="11"/>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B54" s="11" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C54" s="11" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D54" s="11">
         <v>0.4</v>
       </c>
       <c r="E54" s="11"/>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B55" s="11" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C55" s="11" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D55" s="11">
         <v>0.4</v>
       </c>
       <c r="E55" s="11"/>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B56" s="11" t="s">
-        <v>183</v>
+        <v>226</v>
       </c>
       <c r="C56" s="11" t="s">
-        <v>187</v>
+        <v>231</v>
       </c>
       <c r="D56" s="11">
-        <v>11.4</v>
+        <v>0.4</v>
       </c>
       <c r="E56" s="11"/>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B57" s="11" t="s">
-        <v>183</v>
+        <v>226</v>
       </c>
       <c r="C57" s="11" t="s">
-        <v>185</v>
+        <v>232</v>
       </c>
       <c r="D57" s="11">
-        <v>11.4</v>
+        <v>0.4</v>
       </c>
       <c r="E57" s="11"/>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C58" s="11" t="s">
         <v>186</v>
@@ -2840,12 +2889,12 @@
       </c>
       <c r="E58" s="11"/>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" s="11" t="s">
-        <v>8</v>
+        <v>166</v>
       </c>
       <c r="B59" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C59" s="11" t="s">
         <v>184</v>
@@ -2855,252 +2904,325 @@
       </c>
       <c r="E59" s="11"/>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A60" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="B60" s="17" t="s">
-        <v>163</v>
-      </c>
-      <c r="C60" s="18" t="s">
-        <v>165</v>
-      </c>
-      <c r="D60" s="19">
-        <v>0.13500000000000001</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A61" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="B61" s="17" t="s">
-        <v>164</v>
-      </c>
-      <c r="C61" s="18" t="s">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A60" s="11" t="s">
         <v>166</v>
       </c>
-      <c r="D61" s="19">
-        <v>0.23</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B60" s="11" t="s">
+        <v>182</v>
+      </c>
+      <c r="C60" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="D60" s="11">
+        <v>11.4</v>
+      </c>
+      <c r="E60" s="11"/>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A61" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B61" s="11" t="s">
+        <v>182</v>
+      </c>
+      <c r="C61" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="D61" s="11">
+        <v>11.4</v>
+      </c>
+      <c r="E61" s="11"/>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="B62" s="19" t="s">
-        <v>205</v>
+      <c r="B62" s="17" t="s">
+        <v>162</v>
       </c>
       <c r="C62" s="18" t="s">
-        <v>211</v>
+        <v>164</v>
       </c>
       <c r="D62" s="19">
-        <v>2018.3</v>
-      </c>
-      <c r="E62" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.13500000000000001</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="B63" s="19" t="s">
-        <v>206</v>
+      <c r="B63" s="17" t="s">
+        <v>163</v>
       </c>
       <c r="C63" s="18" t="s">
-        <v>213</v>
+        <v>165</v>
       </c>
       <c r="D63" s="19">
-        <v>2022.15</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.23</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" s="17" t="s">
         <v>6</v>
       </c>
       <c r="B64" s="19" t="s">
-        <v>224</v>
+        <v>204</v>
       </c>
       <c r="C64" s="18" t="s">
-        <v>225</v>
+        <v>210</v>
       </c>
       <c r="D64" s="19">
-        <v>2011</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+        <v>2018.3</v>
+      </c>
+      <c r="E64" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" s="17" t="s">
         <v>6</v>
       </c>
       <c r="B65" s="19" t="s">
-        <v>234</v>
+        <v>205</v>
       </c>
       <c r="C65" s="18" t="s">
-        <v>235</v>
+        <v>212</v>
       </c>
       <c r="D65" s="19">
-        <v>2015.3</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+        <v>2022.15</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" s="17" t="s">
         <v>6</v>
       </c>
       <c r="B66" s="19" t="s">
-        <v>207</v>
+        <v>223</v>
       </c>
       <c r="C66" s="18" t="s">
-        <v>210</v>
+        <v>224</v>
       </c>
       <c r="D66" s="19">
-        <v>2024.3</v>
-      </c>
-      <c r="E66" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+        <v>2011</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" s="17" t="s">
         <v>6</v>
       </c>
       <c r="B67" s="19" t="s">
-        <v>214</v>
+        <v>233</v>
       </c>
       <c r="C67" s="18" t="s">
-        <v>212</v>
+        <v>234</v>
       </c>
       <c r="D67" s="19">
-        <v>2040</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+        <v>2015.3</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" s="17" t="s">
         <v>6</v>
       </c>
       <c r="B68" s="19" t="s">
+        <v>206</v>
+      </c>
+      <c r="C68" s="18" t="s">
+        <v>209</v>
+      </c>
+      <c r="D68" s="19">
+        <v>2024.3</v>
+      </c>
+      <c r="E68" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A69" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="B69" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="C69" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="D69" s="19">
+        <v>2040</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A70" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="B70" s="19" t="s">
+        <v>227</v>
+      </c>
+      <c r="C70" s="18" t="s">
         <v>228</v>
       </c>
-      <c r="C68" s="18" t="s">
-        <v>229</v>
-      </c>
-      <c r="D68" s="19">
+      <c r="D70" s="19">
         <v>2040</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A69" t="s">
-        <v>11</v>
-      </c>
-      <c r="B69" t="s">
-        <v>15</v>
-      </c>
-      <c r="C69" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="D69" s="7">
-        <v>0.27033795990919401</v>
-      </c>
-      <c r="E69" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A70" t="s">
-        <v>11</v>
-      </c>
-      <c r="B70" t="s">
-        <v>17</v>
-      </c>
-      <c r="C70" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D70" s="7">
-        <v>8.0685220845966698E-3</v>
-      </c>
-      <c r="E70" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A71" t="s">
-        <v>11</v>
-      </c>
-      <c r="B71" t="s">
-        <v>16</v>
-      </c>
-      <c r="C71" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="D71" s="7">
-        <v>0</v>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A71" s="17" t="s">
+        <v>273</v>
+      </c>
+      <c r="B71" s="19" t="s">
+        <v>274</v>
+      </c>
+      <c r="C71" s="19" t="s">
+        <v>272</v>
+      </c>
+      <c r="D71" s="19">
+        <v>3000</v>
       </c>
       <c r="E71" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A72" t="s">
-        <v>11</v>
-      </c>
-      <c r="B72" t="s">
-        <v>10</v>
-      </c>
-      <c r="C72" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="D72" s="7">
-        <v>0.04</v>
+        <v>119</v>
+      </c>
+      <c r="F71" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A72" s="17" t="s">
+        <v>273</v>
+      </c>
+      <c r="B72" s="19" t="s">
+        <v>275</v>
+      </c>
+      <c r="C72" s="19" t="s">
+        <v>276</v>
+      </c>
+      <c r="D72" s="19">
+        <v>50</v>
       </c>
       <c r="E72" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+        <v>261</v>
+      </c>
+      <c r="F72" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>11</v>
       </c>
       <c r="B73" t="s">
-        <v>222</v>
-      </c>
-      <c r="C73" s="20" t="s">
-        <v>12</v>
+        <v>15</v>
+      </c>
+      <c r="C73" s="7" t="s">
+        <v>120</v>
       </c>
       <c r="D73" s="7">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.27033795990919401</v>
+      </c>
+      <c r="E73" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>11</v>
       </c>
       <c r="B74" t="s">
-        <v>226</v>
-      </c>
-      <c r="C74" s="20" t="s">
-        <v>223</v>
+        <v>17</v>
+      </c>
+      <c r="C74" s="7" t="s">
+        <v>13</v>
       </c>
       <c r="D74" s="7">
-        <v>2000</v>
+        <v>8.0685220845966698E-3</v>
       </c>
       <c r="E74" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>11</v>
       </c>
       <c r="B75" t="s">
+        <v>16</v>
+      </c>
+      <c r="C75" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D75" s="7">
+        <v>0</v>
+      </c>
+      <c r="E75" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>11</v>
+      </c>
+      <c r="B76" t="s">
+        <v>10</v>
+      </c>
+      <c r="C76" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="D76" s="7">
+        <v>0.04</v>
+      </c>
+      <c r="E76" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>11</v>
+      </c>
+      <c r="B77" t="s">
+        <v>221</v>
+      </c>
+      <c r="C77" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D77" s="7">
+        <v>0.8</v>
+      </c>
+      <c r="E77" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>11</v>
+      </c>
+      <c r="B78" t="s">
+        <v>225</v>
+      </c>
+      <c r="C78" s="20" t="s">
+        <v>222</v>
+      </c>
+      <c r="D78" s="7">
+        <v>2000</v>
+      </c>
+      <c r="E78" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>11</v>
+      </c>
+      <c r="B79" t="s">
+        <v>265</v>
+      </c>
+      <c r="C79" s="20" t="s">
         <v>266</v>
       </c>
-      <c r="C75" s="20" t="s">
-        <v>267</v>
-      </c>
-      <c r="D75" s="7">
+      <c r="D79" s="7">
         <v>0.5</v>
       </c>
-      <c r="E75" t="s">
-        <v>203</v>
+      <c r="E79" t="s">
+        <v>202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
warmer homes algorithm fix
</commit_message>
<xml_diff>
--- a/inst/extdata/scenario_parameters.xlsx
+++ b/inst/extdata/scenario_parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joe\pkgs\hpmicrosimr\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A90197CF-AE51-4833-8BA9-7512E9C5CD52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{951385C3-CE04-4B1F-9D61-06FB59178B1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24" yWindow="252" windowWidth="23016" windowHeight="12216" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="24" yWindow="24" windowWidth="23016" windowHeight="12216" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Description" sheetId="7" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="304">
   <si>
     <t>category</t>
   </si>
@@ -1042,6 +1042,18 @@
   </si>
   <si>
     <t>sigma.</t>
+  </si>
+  <si>
+    <t>warmer homes economy of scale factor</t>
+  </si>
+  <si>
+    <t>assume 20% discount to private market</t>
+  </si>
+  <si>
+    <t>warmer_homes_cost_scale</t>
+  </si>
+  <si>
+    <t>B3  in practice</t>
   </si>
 </sst>
 </file>
@@ -1969,7 +1981,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C8E1679-ADB0-42D7-8103-5D0EB0C9F50E}">
-  <dimension ref="A1:F86"/>
+  <dimension ref="A1:F87"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -3150,10 +3162,13 @@
         <v>281</v>
       </c>
       <c r="D71" s="19">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="E71" s="19" t="s">
         <v>258</v>
+      </c>
+      <c r="F71" s="19" t="s">
+        <v>303</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
@@ -3233,23 +3248,20 @@
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A77" s="23" t="s">
-        <v>270</v>
-      </c>
-      <c r="B77" s="24" t="s">
-        <v>271</v>
-      </c>
-      <c r="C77" s="24" t="s">
-        <v>269</v>
-      </c>
-      <c r="D77" s="24">
-        <v>3000</v>
+      <c r="A77" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="B77" s="19" t="s">
+        <v>300</v>
+      </c>
+      <c r="C77" s="19" t="s">
+        <v>302</v>
+      </c>
+      <c r="D77" s="19">
+        <v>0.8</v>
       </c>
       <c r="E77" t="s">
-        <v>119</v>
-      </c>
-      <c r="F77" t="s">
-        <v>274</v>
+        <v>301</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
@@ -3257,36 +3269,39 @@
         <v>270</v>
       </c>
       <c r="B78" s="24" t="s">
+        <v>271</v>
+      </c>
+      <c r="C78" s="24" t="s">
+        <v>269</v>
+      </c>
+      <c r="D78" s="24">
+        <v>3000</v>
+      </c>
+      <c r="E78" t="s">
+        <v>119</v>
+      </c>
+      <c r="F78" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A79" s="23" t="s">
+        <v>270</v>
+      </c>
+      <c r="B79" s="24" t="s">
         <v>272</v>
       </c>
-      <c r="C78" s="24" t="s">
+      <c r="C79" s="24" t="s">
         <v>273</v>
       </c>
-      <c r="D78" s="24">
+      <c r="D79" s="24">
         <v>50</v>
       </c>
-      <c r="E78" t="s">
+      <c r="E79" t="s">
         <v>258</v>
       </c>
-      <c r="F78" t="s">
+      <c r="F79" t="s">
         <v>275</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A79" t="s">
-        <v>11</v>
-      </c>
-      <c r="B79" t="s">
-        <v>15</v>
-      </c>
-      <c r="C79" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="D79" s="7">
-        <v>0.15</v>
-      </c>
-      <c r="E79" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
@@ -3294,13 +3309,13 @@
         <v>11</v>
       </c>
       <c r="B80" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C80" s="7" t="s">
-        <v>13</v>
+        <v>120</v>
       </c>
       <c r="D80" s="7">
-        <v>2.2000000000000001E-3</v>
+        <v>0.15</v>
       </c>
       <c r="E80" t="s">
         <v>121</v>
@@ -3311,16 +3326,16 @@
         <v>11</v>
       </c>
       <c r="B81" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C81" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D81" s="7">
-        <v>0</v>
+        <v>2.2000000000000001E-3</v>
       </c>
       <c r="E81" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
@@ -3328,16 +3343,16 @@
         <v>11</v>
       </c>
       <c r="B82" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C82" s="7" t="s">
-        <v>263</v>
+        <v>14</v>
       </c>
       <c r="D82" s="7">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="E82" t="s">
-        <v>268</v>
+        <v>122</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
@@ -3345,16 +3360,16 @@
         <v>11</v>
       </c>
       <c r="B83" t="s">
-        <v>220</v>
-      </c>
-      <c r="C83" s="20" t="s">
-        <v>12</v>
+        <v>10</v>
+      </c>
+      <c r="C83" s="7" t="s">
+        <v>263</v>
       </c>
       <c r="D83" s="7">
-        <v>0.8</v>
+        <v>0.04</v>
       </c>
       <c r="E83" t="s">
-        <v>201</v>
+        <v>268</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
@@ -3362,16 +3377,16 @@
         <v>11</v>
       </c>
       <c r="B84" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C84" s="20" t="s">
-        <v>285</v>
+        <v>12</v>
       </c>
       <c r="D84" s="7">
         <v>0.8</v>
       </c>
       <c r="E84" t="s">
-        <v>286</v>
+        <v>201</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
@@ -3379,19 +3394,16 @@
         <v>11</v>
       </c>
       <c r="B85" t="s">
-        <v>262</v>
+        <v>223</v>
       </c>
       <c r="C85" s="20" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D85" s="7">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="E85" t="s">
-        <v>201</v>
-      </c>
-      <c r="F85" s="22">
-        <v>0.3</v>
+        <v>286</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
@@ -3399,15 +3411,35 @@
         <v>11</v>
       </c>
       <c r="B86" t="s">
+        <v>262</v>
+      </c>
+      <c r="C86" s="20" t="s">
+        <v>284</v>
+      </c>
+      <c r="D86" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="E86" t="s">
+        <v>201</v>
+      </c>
+      <c r="F86" s="22">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>11</v>
+      </c>
+      <c r="B87" t="s">
         <v>298</v>
       </c>
-      <c r="C86" s="20" t="s">
+      <c r="C87" s="20" t="s">
         <v>299</v>
       </c>
-      <c r="D86" s="7">
+      <c r="D87" s="7">
         <v>0.1</v>
       </c>
-      <c r="E86" t="s">
+      <c r="E87" t="s">
         <v>201</v>
       </c>
     </row>

</xml_diff>

<commit_message>
warmer homes capex cap
</commit_message>
<xml_diff>
--- a/inst/extdata/scenario_parameters.xlsx
+++ b/inst/extdata/scenario_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joe\pkgs\hpmicrosimr\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FE784C7-D01A-46BE-8506-146056EFB7CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A9D47C9-9C63-4883-A578-DEFA75CD93FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="24" yWindow="24" windowWidth="23016" windowHeight="12216" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1091" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1096" uniqueCount="242">
   <si>
     <t>category</t>
   </si>
@@ -757,6 +757,15 @@
   </si>
   <si>
     <t>minimum_fabric_grant</t>
+  </si>
+  <si>
+    <t>Warmer Homes cost cap</t>
+  </si>
+  <si>
+    <t>lag effect (2 years)</t>
+  </si>
+  <si>
+    <t>warmer_homes_cost_cap</t>
   </si>
 </sst>
 </file>
@@ -1325,7 +1334,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C8E1679-ADB0-42D7-8103-5D0EB0C9F50E}">
-  <dimension ref="A1:F93"/>
+  <dimension ref="A1:F94"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -2593,30 +2602,37 @@
         <v>6</v>
       </c>
       <c r="B74" s="14" t="s">
-        <v>177</v>
+        <v>239</v>
       </c>
       <c r="C74" s="13" t="s">
-        <v>179</v>
+        <v>241</v>
       </c>
       <c r="D74" s="14">
-        <v>2025</v>
+        <v>35000</v>
       </c>
       <c r="E74" s="14" t="s">
-        <v>180</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="F74" s="14"/>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" s="12" t="s">
         <v>6</v>
       </c>
       <c r="B75" s="14" t="s">
-        <v>128</v>
+        <v>177</v>
       </c>
       <c r="C75" s="13" t="s">
-        <v>129</v>
+        <v>179</v>
       </c>
       <c r="D75" s="14">
-        <v>2015.3</v>
+        <v>2027</v>
+      </c>
+      <c r="E75" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="F75" s="14" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
@@ -2624,16 +2640,13 @@
         <v>6</v>
       </c>
       <c r="B76" s="14" t="s">
-        <v>102</v>
+        <v>128</v>
       </c>
       <c r="C76" s="13" t="s">
-        <v>105</v>
+        <v>129</v>
       </c>
       <c r="D76" s="14">
-        <v>2024.3</v>
-      </c>
-      <c r="E76" t="s">
-        <v>104</v>
+        <v>2015.3</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
@@ -2641,13 +2654,16 @@
         <v>6</v>
       </c>
       <c r="B77" s="14" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="C77" s="13" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D77" s="14">
-        <v>2040</v>
+        <v>2024.3</v>
+      </c>
+      <c r="E77" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
@@ -2655,10 +2671,10 @@
         <v>6</v>
       </c>
       <c r="B78" s="14" t="s">
-        <v>122</v>
+        <v>109</v>
       </c>
       <c r="C78" s="13" t="s">
-        <v>123</v>
+        <v>107</v>
       </c>
       <c r="D78" s="14">
         <v>2040</v>
@@ -2669,16 +2685,13 @@
         <v>6</v>
       </c>
       <c r="B79" s="14" t="s">
-        <v>197</v>
-      </c>
-      <c r="C79" s="14" t="s">
-        <v>199</v>
+        <v>122</v>
+      </c>
+      <c r="C79" s="13" t="s">
+        <v>123</v>
       </c>
       <c r="D79" s="14">
-        <v>0.8</v>
-      </c>
-      <c r="E79" t="s">
-        <v>198</v>
+        <v>2040</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
@@ -2686,16 +2699,16 @@
         <v>6</v>
       </c>
       <c r="B80" s="14" t="s">
-        <v>233</v>
+        <v>197</v>
       </c>
       <c r="C80" s="14" t="s">
-        <v>230</v>
+        <v>199</v>
       </c>
       <c r="D80" s="14">
-        <v>63.5</v>
+        <v>0.8</v>
       </c>
       <c r="E80" t="s">
-        <v>236</v>
+        <v>198</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
@@ -2703,13 +2716,13 @@
         <v>6</v>
       </c>
       <c r="B81" s="14" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C81" s="14" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D81" s="14">
-        <v>100</v>
+        <v>63.5</v>
       </c>
       <c r="E81" t="s">
         <v>236</v>
@@ -2720,36 +2733,33 @@
         <v>6</v>
       </c>
       <c r="B82" s="14" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C82" s="14" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D82" s="14">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="E82" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A83" s="18" t="s">
-        <v>167</v>
-      </c>
-      <c r="B83" s="19" t="s">
-        <v>168</v>
-      </c>
-      <c r="C83" s="19" t="s">
-        <v>166</v>
-      </c>
-      <c r="D83" s="19">
-        <v>3000</v>
+      <c r="A83" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B83" s="14" t="s">
+        <v>235</v>
+      </c>
+      <c r="C83" s="14" t="s">
+        <v>232</v>
+      </c>
+      <c r="D83" s="14">
+        <v>200</v>
       </c>
       <c r="E83" t="s">
-        <v>23</v>
-      </c>
-      <c r="F83" t="s">
-        <v>171</v>
+        <v>236</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
@@ -2757,36 +2767,39 @@
         <v>167</v>
       </c>
       <c r="B84" s="19" t="s">
+        <v>168</v>
+      </c>
+      <c r="C84" s="19" t="s">
+        <v>166</v>
+      </c>
+      <c r="D84" s="19">
+        <v>3000</v>
+      </c>
+      <c r="E84" t="s">
+        <v>23</v>
+      </c>
+      <c r="F84" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A85" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="B85" s="19" t="s">
         <v>169</v>
       </c>
-      <c r="C84" s="19" t="s">
+      <c r="C85" s="19" t="s">
         <v>170</v>
       </c>
-      <c r="D84" s="19">
+      <c r="D85" s="19">
         <v>50</v>
       </c>
-      <c r="E84" t="s">
+      <c r="E85" t="s">
         <v>155</v>
       </c>
-      <c r="F84" t="s">
+      <c r="F85" t="s">
         <v>172</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A85" t="s">
-        <v>11</v>
-      </c>
-      <c r="B85" t="s">
-        <v>15</v>
-      </c>
-      <c r="C85" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D85" s="3">
-        <v>0.15</v>
-      </c>
-      <c r="E85" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
@@ -2794,13 +2807,13 @@
         <v>11</v>
       </c>
       <c r="B86" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="D86" s="3">
-        <v>2.2000000000000001E-3</v>
+        <v>0.15</v>
       </c>
       <c r="E86" t="s">
         <v>25</v>
@@ -2811,16 +2824,16 @@
         <v>11</v>
       </c>
       <c r="B87" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D87" s="3">
-        <v>0</v>
+        <v>2.2000000000000001E-3</v>
       </c>
       <c r="E87" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
@@ -2828,16 +2841,16 @@
         <v>11</v>
       </c>
       <c r="B88" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>160</v>
+        <v>14</v>
       </c>
       <c r="D88" s="3">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="E88" t="s">
-        <v>165</v>
+        <v>26</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
@@ -2845,16 +2858,16 @@
         <v>11</v>
       </c>
       <c r="B89" t="s">
-        <v>117</v>
-      </c>
-      <c r="C89" s="15" t="s">
-        <v>12</v>
+        <v>10</v>
+      </c>
+      <c r="C89" s="3" t="s">
+        <v>160</v>
       </c>
       <c r="D89" s="3">
-        <v>0.8</v>
+        <v>0.04</v>
       </c>
       <c r="E89" t="s">
-        <v>98</v>
+        <v>165</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
@@ -2862,19 +2875,16 @@
         <v>11</v>
       </c>
       <c r="B90" t="s">
-        <v>209</v>
+        <v>117</v>
       </c>
       <c r="C90" s="15" t="s">
-        <v>182</v>
+        <v>12</v>
       </c>
       <c r="D90" s="3">
-        <v>0.02</v>
+        <v>0.8</v>
       </c>
       <c r="E90" t="s">
         <v>98</v>
-      </c>
-      <c r="F90" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
@@ -2882,19 +2892,19 @@
         <v>11</v>
       </c>
       <c r="B91" t="s">
-        <v>159</v>
+        <v>209</v>
       </c>
       <c r="C91" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D91" s="3">
-        <v>0.3</v>
+        <v>0.02</v>
       </c>
       <c r="E91" t="s">
         <v>98</v>
       </c>
-      <c r="F91" s="17">
-        <v>0.3</v>
+      <c r="F91" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
@@ -2902,16 +2912,19 @@
         <v>11</v>
       </c>
       <c r="B92" t="s">
-        <v>195</v>
+        <v>159</v>
       </c>
       <c r="C92" s="15" t="s">
-        <v>196</v>
+        <v>181</v>
       </c>
       <c r="D92" s="3">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="E92" t="s">
         <v>98</v>
+      </c>
+      <c r="F92" s="17">
+        <v>0.3</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
@@ -2919,18 +2932,35 @@
         <v>11</v>
       </c>
       <c r="B93" t="s">
-        <v>213</v>
+        <v>195</v>
       </c>
       <c r="C93" s="15" t="s">
-        <v>211</v>
+        <v>196</v>
       </c>
       <c r="D93" s="3">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="E93" t="s">
         <v>98</v>
       </c>
-      <c r="F93" t="s">
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A94" t="s">
+        <v>11</v>
+      </c>
+      <c r="B94" t="s">
+        <v>213</v>
+      </c>
+      <c r="C94" s="15" t="s">
+        <v>211</v>
+      </c>
+      <c r="D94" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="E94" t="s">
+        <v>98</v>
+      </c>
+      <c r="F94" t="s">
         <v>212</v>
       </c>
     </row>

</xml_diff>

<commit_message>
2040 heat pump efficiency added
</commit_message>
<xml_diff>
--- a/inst/extdata/scenario_parameters.xlsx
+++ b/inst/extdata/scenario_parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joe\pkgs\hpmicrosimr\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{129330EA-8F45-476A-8481-5A2561AFD5E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C339CC27-54AB-48B5-B03E-7DCB3C71AC21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24" yWindow="48" windowWidth="23016" windowHeight="12216" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="24" yWindow="744" windowWidth="23016" windowHeight="12216" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Description" sheetId="7" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1152" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1156" uniqueCount="251">
   <si>
     <t>category</t>
   </si>
@@ -790,6 +790,9 @@
   </si>
   <si>
     <t>grant_increase_factor</t>
+  </si>
+  <si>
+    <t>heat_pump_cop_2040</t>
   </si>
 </sst>
 </file>
@@ -3046,7 +3049,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BA1BE81-9C4C-49AE-A7FD-599BD867D62D}">
-  <dimension ref="A1:F97"/>
+  <dimension ref="A1:F98"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="57.88671875" customWidth="1"/>
@@ -3469,19 +3472,16 @@
         <v>18</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>137</v>
+        <v>44</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>138</v>
+        <v>250</v>
       </c>
       <c r="D24" s="6">
-        <v>0.6</v>
+        <v>3.25</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>98</v>
-      </c>
-      <c r="F24" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
@@ -3492,16 +3492,16 @@
         <v>137</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D25" s="6">
-        <v>0.85</v>
+        <v>0.6</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>98</v>
       </c>
       <c r="F25" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
@@ -3512,13 +3512,16 @@
         <v>137</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D26" s="6">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>98</v>
+      </c>
+      <c r="F26" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
@@ -3526,50 +3529,50 @@
         <v>18</v>
       </c>
       <c r="B27" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="D27" s="6">
+        <v>0.9</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B28" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C28" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="D27" s="6">
+      <c r="D28" s="6">
         <v>0.75</v>
       </c>
-      <c r="E27" s="6" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B28" s="10" t="s">
-        <v>85</v>
-      </c>
-      <c r="C28" s="10" t="s">
-        <v>149</v>
-      </c>
-      <c r="D28" s="10">
-        <v>1</v>
-      </c>
-      <c r="E28" s="10" t="s">
+      <c r="E28" s="6" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="10" t="s">
-        <v>56</v>
+        <v>18</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>46</v>
+        <v>149</v>
       </c>
       <c r="D29" s="10">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>9</v>
+        <v>98</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
@@ -3577,13 +3580,13 @@
         <v>56</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D30" s="10">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E30" s="10" t="s">
         <v>9</v>
@@ -3594,13 +3597,13 @@
         <v>56</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="D31" s="10">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E31" s="10" t="s">
         <v>9</v>
@@ -3611,13 +3614,13 @@
         <v>56</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="D32" s="10">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E32" s="10" t="s">
         <v>9</v>
@@ -3628,13 +3631,13 @@
         <v>56</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>87</v>
+        <v>50</v>
       </c>
       <c r="D33" s="10">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="E33" s="10" t="s">
         <v>9</v>
@@ -3645,16 +3648,16 @@
         <v>56</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>129</v>
+        <v>52</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>130</v>
+        <v>87</v>
       </c>
       <c r="D34" s="10">
-        <v>2.5</v>
-      </c>
-      <c r="E34" s="6" t="s">
-        <v>98</v>
+        <v>25</v>
+      </c>
+      <c r="E34" s="10" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
@@ -3662,10 +3665,10 @@
         <v>56</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D35" s="10">
         <v>2.5</v>
@@ -3679,13 +3682,13 @@
         <v>56</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D36" s="10">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>98</v>
@@ -3696,50 +3699,50 @@
         <v>56</v>
       </c>
       <c r="B37" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="C37" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="D37" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B38" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="C37" s="10" t="s">
+      <c r="C38" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="D37" s="10">
+      <c r="D38" s="10">
         <v>3</v>
       </c>
-      <c r="E37" s="6" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="B38" s="16" t="s">
-        <v>145</v>
-      </c>
-      <c r="C38" s="16" t="s">
-        <v>144</v>
-      </c>
-      <c r="D38" s="16">
-        <v>2</v>
-      </c>
-      <c r="E38" s="16" t="s">
+      <c r="E38" s="6" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="16" t="s">
-        <v>18</v>
+        <v>56</v>
       </c>
       <c r="B39" s="16" t="s">
-        <v>183</v>
+        <v>145</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="D39" s="16">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="E39" s="16" t="s">
-        <v>154</v>
+        <v>98</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
@@ -3747,13 +3750,13 @@
         <v>18</v>
       </c>
       <c r="B40" s="16" t="s">
-        <v>155</v>
+        <v>183</v>
       </c>
       <c r="C40" s="16" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="D40" s="16">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="E40" s="16" t="s">
         <v>154</v>
@@ -3764,13 +3767,13 @@
         <v>18</v>
       </c>
       <c r="B41" s="16" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C41" s="16" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="D41" s="16">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="E41" s="16" t="s">
         <v>154</v>
@@ -3781,19 +3784,16 @@
         <v>18</v>
       </c>
       <c r="B42" s="16" t="s">
-        <v>182</v>
+        <v>156</v>
       </c>
       <c r="C42" s="16" t="s">
-        <v>184</v>
+        <v>157</v>
       </c>
       <c r="D42" s="16">
-        <v>2.2999999999999998</v>
+        <v>8</v>
       </c>
       <c r="E42" s="16" t="s">
-        <v>185</v>
-      </c>
-      <c r="F42" t="s">
-        <v>186</v>
+        <v>154</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
@@ -3801,28 +3801,33 @@
         <v>18</v>
       </c>
       <c r="B43" s="16" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C43" s="16" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="D43" s="16">
-        <v>1.25</v>
-      </c>
-      <c r="E43" s="16"/>
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="E43" s="16" t="s">
+        <v>185</v>
+      </c>
+      <c r="F43" t="s">
+        <v>186</v>
+      </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="16" t="s">
         <v>18</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D44" s="16">
-        <v>1.1000000000000001</v>
+        <v>1.25</v>
       </c>
       <c r="E44" s="16"/>
     </row>
@@ -3831,13 +3836,13 @@
         <v>18</v>
       </c>
       <c r="B45" s="16" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C45" s="16" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D45" s="16">
-        <v>1.08</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="E45" s="16"/>
     </row>
@@ -3846,56 +3851,54 @@
         <v>18</v>
       </c>
       <c r="B46" s="16" t="s">
+        <v>189</v>
+      </c>
+      <c r="C46" s="16" t="s">
+        <v>192</v>
+      </c>
+      <c r="D46" s="16">
+        <v>1.08</v>
+      </c>
+      <c r="E46" s="16"/>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="B47" s="16" t="s">
         <v>240</v>
       </c>
-      <c r="C46" s="16" t="s">
+      <c r="C47" s="16" t="s">
         <v>241</v>
       </c>
-      <c r="D46" s="16">
+      <c r="D47" s="16">
         <v>0.3</v>
       </c>
-      <c r="E46" s="16" t="s">
-        <v>98</v>
-      </c>
-      <c r="F46" s="16" t="s">
+      <c r="E47" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="F47" s="16" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="11" t="s">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B47" s="11" t="s">
+      <c r="B48" s="11" t="s">
         <v>150</v>
       </c>
-      <c r="C47" s="11" t="s">
+      <c r="C48" s="11" t="s">
         <v>242</v>
       </c>
-      <c r="D47" s="11">
+      <c r="D48" s="11">
         <v>0.6</v>
       </c>
-      <c r="E47" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="F47" s="10" t="s">
+      <c r="E48" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="F48" s="10" t="s">
         <v>243</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="B48" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C48" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="D48" s="6">
-        <v>11.8</v>
-      </c>
-      <c r="E48" s="6" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -3903,19 +3906,16 @@
         <v>62</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>63</v>
+        <v>99</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D49" s="6">
-        <v>12.8</v>
+        <v>11.8</v>
       </c>
       <c r="E49" s="6" t="s">
         <v>199</v>
-      </c>
-      <c r="F49" s="6" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
@@ -3926,13 +3926,16 @@
         <v>63</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D50" s="6">
-        <v>13.8</v>
+        <v>12.8</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>199</v>
+      </c>
+      <c r="F50" s="6" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
@@ -3943,10 +3946,10 @@
         <v>63</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D51" s="6">
-        <v>16.8</v>
+        <v>13.8</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>199</v>
@@ -3957,13 +3960,13 @@
         <v>62</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D52" s="6">
-        <v>13.2</v>
+        <v>16.8</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>199</v>
@@ -3977,16 +3980,13 @@
         <v>68</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D53" s="6">
-        <v>14</v>
+        <v>13.2</v>
       </c>
       <c r="E53" s="6" t="s">
         <v>199</v>
-      </c>
-      <c r="F53" s="6" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
@@ -3997,13 +3997,16 @@
         <v>68</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D54" s="6">
-        <v>14.8</v>
+        <v>14</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>199</v>
+      </c>
+      <c r="F54" s="6" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
@@ -4014,10 +4017,10 @@
         <v>68</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D55" s="6">
-        <v>17.2</v>
+        <v>14.8</v>
       </c>
       <c r="E55" s="6" t="s">
         <v>199</v>
@@ -4028,18 +4031,17 @@
         <v>62</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D56" s="6">
-        <v>35.4</v>
+        <v>17.2</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="F56" s="6"/>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="6" t="s">
@@ -4049,7 +4051,7 @@
         <v>73</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D57" s="6">
         <v>35.4</v>
@@ -4057,6 +4059,7 @@
       <c r="E57" s="6" t="s">
         <v>199</v>
       </c>
+      <c r="F57" s="6"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="6" t="s">
@@ -4066,7 +4069,7 @@
         <v>73</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D58" s="6">
         <v>35.4</v>
@@ -4083,7 +4086,7 @@
         <v>73</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D59" s="6">
         <v>35.4</v>
@@ -4097,15 +4100,17 @@
         <v>62</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>120</v>
+        <v>73</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>123</v>
+        <v>77</v>
       </c>
       <c r="D60" s="6">
-        <v>0.4</v>
-      </c>
-      <c r="E60" s="6"/>
+        <v>35.4</v>
+      </c>
+      <c r="E60" s="6" t="s">
+        <v>199</v>
+      </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" s="6" t="s">
@@ -4115,7 +4120,7 @@
         <v>120</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D61" s="6">
         <v>0.4</v>
@@ -4130,7 +4135,7 @@
         <v>120</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D62" s="6">
         <v>0.4</v>
@@ -4145,7 +4150,7 @@
         <v>120</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D63" s="6">
         <v>0.4</v>
@@ -4157,18 +4162,15 @@
         <v>62</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>78</v>
+        <v>120</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>82</v>
+        <v>126</v>
       </c>
       <c r="D64" s="6">
-        <v>11.4</v>
+        <v>0.4</v>
       </c>
       <c r="E64" s="6"/>
-      <c r="F64" s="6" t="s">
-        <v>202</v>
-      </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" s="6" t="s">
@@ -4178,14 +4180,14 @@
         <v>78</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D65" s="6">
-        <v>12.7</v>
+        <v>11.4</v>
       </c>
       <c r="E65" s="6"/>
       <c r="F65" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
@@ -4196,57 +4198,61 @@
         <v>78</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D66" s="6">
-        <v>14</v>
+        <v>12.7</v>
       </c>
       <c r="E66" s="6"/>
+      <c r="F66" s="6" t="s">
+        <v>203</v>
+      </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" s="6" t="s">
-        <v>8</v>
+        <v>62</v>
       </c>
       <c r="B67" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C67" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="D67" s="6">
+        <v>14</v>
+      </c>
+      <c r="E67" s="6"/>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A68" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B68" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C68" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="D67" s="6">
+      <c r="D68" s="6">
         <v>17.899999999999999</v>
       </c>
-      <c r="E67" s="6"/>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A68" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="B68" s="12" t="s">
-        <v>235</v>
-      </c>
-      <c r="C68" s="13" t="s">
-        <v>236</v>
-      </c>
-      <c r="D68" s="14">
-        <v>700</v>
-      </c>
-      <c r="E68" t="s">
-        <v>7</v>
-      </c>
+      <c r="E68" s="6"/>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" s="12" t="s">
         <v>6</v>
       </c>
       <c r="B69" s="12" t="s">
-        <v>58</v>
+        <v>235</v>
       </c>
       <c r="C69" s="13" t="s">
-        <v>60</v>
+        <v>236</v>
       </c>
       <c r="D69" s="14">
-        <v>0.13500000000000001</v>
+        <v>700</v>
+      </c>
+      <c r="E69" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
@@ -4254,30 +4260,27 @@
         <v>6</v>
       </c>
       <c r="B70" s="12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C70" s="13" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D70" s="14">
-        <v>0.23</v>
+        <v>0.13500000000000001</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B71" s="14" t="s">
-        <v>100</v>
+      <c r="B71" s="12" t="s">
+        <v>59</v>
       </c>
       <c r="C71" s="13" t="s">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="D71" s="14">
-        <v>2018.3</v>
-      </c>
-      <c r="E71" t="s">
-        <v>103</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
@@ -4285,13 +4288,16 @@
         <v>6</v>
       </c>
       <c r="B72" s="14" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C72" s="13" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D72" s="14">
-        <v>2022.15</v>
+        <v>2018.3</v>
+      </c>
+      <c r="E72" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
@@ -4299,13 +4305,13 @@
         <v>6</v>
       </c>
       <c r="B73" s="14" t="s">
-        <v>118</v>
+        <v>101</v>
       </c>
       <c r="C73" s="13" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="D73" s="14">
-        <v>2011</v>
+        <v>2022.15</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
@@ -4313,19 +4319,13 @@
         <v>6</v>
       </c>
       <c r="B74" s="14" t="s">
-        <v>175</v>
+        <v>118</v>
       </c>
       <c r="C74" s="13" t="s">
-        <v>177</v>
+        <v>119</v>
       </c>
       <c r="D74" s="14">
-        <v>150</v>
-      </c>
-      <c r="E74" s="14" t="s">
-        <v>154</v>
-      </c>
-      <c r="F74" s="14" t="s">
-        <v>198</v>
+        <v>2011</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
@@ -4333,51 +4333,57 @@
         <v>6</v>
       </c>
       <c r="B75" s="14" t="s">
-        <v>237</v>
+        <v>175</v>
       </c>
       <c r="C75" s="13" t="s">
-        <v>239</v>
+        <v>177</v>
       </c>
       <c r="D75" s="14">
-        <v>35000</v>
+        <v>150</v>
       </c>
       <c r="E75" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="F75" s="14"/>
+        <v>154</v>
+      </c>
+      <c r="F75" s="14" t="s">
+        <v>198</v>
+      </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" s="12" t="s">
         <v>6</v>
       </c>
       <c r="B76" s="14" t="s">
-        <v>176</v>
+        <v>237</v>
       </c>
       <c r="C76" s="13" t="s">
-        <v>178</v>
+        <v>239</v>
       </c>
       <c r="D76" s="14">
-        <v>2027</v>
+        <v>35000</v>
       </c>
       <c r="E76" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="F76" s="14" t="s">
-        <v>238</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="F76" s="14"/>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" s="12" t="s">
         <v>6</v>
       </c>
       <c r="B77" s="14" t="s">
-        <v>127</v>
+        <v>176</v>
       </c>
       <c r="C77" s="13" t="s">
-        <v>128</v>
+        <v>178</v>
       </c>
       <c r="D77" s="14">
-        <v>2015.3</v>
+        <v>2027</v>
+      </c>
+      <c r="E77" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="F77" s="14" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
@@ -4385,16 +4391,13 @@
         <v>6</v>
       </c>
       <c r="B78" s="14" t="s">
-        <v>102</v>
+        <v>127</v>
       </c>
       <c r="C78" s="13" t="s">
-        <v>105</v>
+        <v>128</v>
       </c>
       <c r="D78" s="14">
-        <v>2024.3</v>
-      </c>
-      <c r="E78" t="s">
-        <v>104</v>
+        <v>2015.3</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
@@ -4402,13 +4405,16 @@
         <v>6</v>
       </c>
       <c r="B79" s="14" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="C79" s="13" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D79" s="14">
-        <v>2040</v>
+        <v>2024.3</v>
+      </c>
+      <c r="E79" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
@@ -4416,10 +4422,10 @@
         <v>6</v>
       </c>
       <c r="B80" s="14" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="C80" s="13" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="D80" s="14">
         <v>2040</v>
@@ -4430,16 +4436,13 @@
         <v>6</v>
       </c>
       <c r="B81" s="14" t="s">
-        <v>195</v>
-      </c>
-      <c r="C81" s="14" t="s">
-        <v>197</v>
+        <v>121</v>
+      </c>
+      <c r="C81" s="13" t="s">
+        <v>122</v>
       </c>
       <c r="D81" s="14">
-        <v>0.8</v>
-      </c>
-      <c r="E81" t="s">
-        <v>196</v>
+        <v>2040</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
@@ -4447,16 +4450,16 @@
         <v>6</v>
       </c>
       <c r="B82" s="14" t="s">
-        <v>231</v>
+        <v>195</v>
       </c>
       <c r="C82" s="14" t="s">
-        <v>228</v>
+        <v>197</v>
       </c>
       <c r="D82" s="14">
-        <v>63.5</v>
+        <v>0.8</v>
       </c>
       <c r="E82" t="s">
-        <v>234</v>
+        <v>196</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
@@ -4464,13 +4467,13 @@
         <v>6</v>
       </c>
       <c r="B83" s="14" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C83" s="14" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D83" s="14">
-        <v>100</v>
+        <v>63.5</v>
       </c>
       <c r="E83" t="s">
         <v>234</v>
@@ -4481,13 +4484,13 @@
         <v>6</v>
       </c>
       <c r="B84" s="14" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C84" s="14" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D84" s="14">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="E84" t="s">
         <v>234</v>
@@ -4498,13 +4501,16 @@
         <v>6</v>
       </c>
       <c r="B85" s="14" t="s">
-        <v>246</v>
+        <v>233</v>
       </c>
       <c r="C85" s="14" t="s">
-        <v>248</v>
+        <v>230</v>
       </c>
       <c r="D85" s="14">
-        <v>2026.5</v>
+        <v>200</v>
+      </c>
+      <c r="E85" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
@@ -4512,33 +4518,27 @@
         <v>6</v>
       </c>
       <c r="B86" s="14" t="s">
+        <v>246</v>
+      </c>
+      <c r="C86" s="14" t="s">
+        <v>248</v>
+      </c>
+      <c r="D86" s="14">
+        <v>2026.5</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A87" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B87" s="14" t="s">
         <v>247</v>
       </c>
-      <c r="C86" s="14" t="s">
+      <c r="C87" s="14" t="s">
         <v>249</v>
       </c>
-      <c r="D86" s="14">
+      <c r="D87" s="14">
         <v>1.5</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A87" s="18" t="s">
-        <v>166</v>
-      </c>
-      <c r="B87" s="19" t="s">
-        <v>167</v>
-      </c>
-      <c r="C87" s="19" t="s">
-        <v>165</v>
-      </c>
-      <c r="D87" s="19">
-        <v>3000</v>
-      </c>
-      <c r="E87" t="s">
-        <v>23</v>
-      </c>
-      <c r="F87" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
@@ -4546,36 +4546,39 @@
         <v>166</v>
       </c>
       <c r="B88" s="19" t="s">
+        <v>167</v>
+      </c>
+      <c r="C88" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="D88" s="19">
+        <v>3000</v>
+      </c>
+      <c r="E88" t="s">
+        <v>23</v>
+      </c>
+      <c r="F88" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A89" s="18" t="s">
+        <v>166</v>
+      </c>
+      <c r="B89" s="19" t="s">
         <v>168</v>
       </c>
-      <c r="C88" s="19" t="s">
+      <c r="C89" s="19" t="s">
         <v>169</v>
       </c>
-      <c r="D88" s="19">
+      <c r="D89" s="19">
         <v>75</v>
       </c>
-      <c r="E88" t="s">
+      <c r="E89" t="s">
         <v>154</v>
       </c>
-      <c r="F88" t="s">
+      <c r="F89" t="s">
         <v>245</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A89" t="s">
-        <v>11</v>
-      </c>
-      <c r="B89" t="s">
-        <v>15</v>
-      </c>
-      <c r="C89" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D89">
-        <v>0.594322503</v>
-      </c>
-      <c r="E89" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
@@ -4583,13 +4586,13 @@
         <v>11</v>
       </c>
       <c r="B90" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="D90">
-        <v>4.8274562E-2</v>
+        <v>0.594322503</v>
       </c>
       <c r="E90" t="s">
         <v>25</v>
@@ -4600,16 +4603,16 @@
         <v>11</v>
       </c>
       <c r="B91" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D91" s="3">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="D91">
+        <v>4.8274562E-2</v>
       </c>
       <c r="E91" t="s">
-        <v>244</v>
+        <v>25</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
@@ -4617,16 +4620,16 @@
         <v>11</v>
       </c>
       <c r="B92" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="D92">
-        <v>0.03</v>
+        <v>14</v>
+      </c>
+      <c r="D92" s="3">
+        <v>0</v>
       </c>
       <c r="E92" t="s">
-        <v>164</v>
+        <v>244</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
@@ -4634,16 +4637,16 @@
         <v>11</v>
       </c>
       <c r="B93" t="s">
-        <v>117</v>
-      </c>
-      <c r="C93" s="15" t="s">
-        <v>12</v>
+        <v>10</v>
+      </c>
+      <c r="C93" s="3" t="s">
+        <v>159</v>
       </c>
       <c r="D93">
-        <v>0.40077507600000001</v>
+        <v>0.03</v>
       </c>
       <c r="E93" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
@@ -4651,19 +4654,16 @@
         <v>11</v>
       </c>
       <c r="B94" t="s">
-        <v>207</v>
+        <v>117</v>
       </c>
       <c r="C94" s="15" t="s">
-        <v>181</v>
+        <v>12</v>
       </c>
       <c r="D94">
-        <v>0.12119928100000001</v>
+        <v>0.40077507600000001</v>
       </c>
       <c r="E94" t="s">
         <v>98</v>
-      </c>
-      <c r="F94" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
@@ -4671,19 +4671,19 @@
         <v>11</v>
       </c>
       <c r="B95" t="s">
-        <v>158</v>
+        <v>207</v>
       </c>
       <c r="C95" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="D95" s="3">
-        <v>0.3</v>
+        <v>181</v>
+      </c>
+      <c r="D95">
+        <v>0.12119928100000001</v>
       </c>
       <c r="E95" t="s">
         <v>98</v>
       </c>
-      <c r="F95" s="17">
-        <v>0.3</v>
+      <c r="F95" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
@@ -4691,16 +4691,19 @@
         <v>11</v>
       </c>
       <c r="B96" t="s">
-        <v>193</v>
+        <v>158</v>
       </c>
       <c r="C96" s="15" t="s">
-        <v>194</v>
+        <v>180</v>
       </c>
       <c r="D96" s="3">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="E96" t="s">
         <v>98</v>
+      </c>
+      <c r="F96" s="17">
+        <v>0.3</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
@@ -4708,18 +4711,35 @@
         <v>11</v>
       </c>
       <c r="B97" t="s">
+        <v>193</v>
+      </c>
+      <c r="C97" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="D97" s="3">
+        <v>0</v>
+      </c>
+      <c r="E97" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
+        <v>11</v>
+      </c>
+      <c r="B98" t="s">
         <v>211</v>
       </c>
-      <c r="C97" s="15" t="s">
+      <c r="C98" s="15" t="s">
         <v>209</v>
       </c>
-      <c r="D97">
+      <c r="D98">
         <v>1.2961873E-2</v>
       </c>
-      <c r="E97" t="s">
-        <v>98</v>
-      </c>
-      <c r="F97" t="s">
+      <c r="E98" t="s">
+        <v>98</v>
+      </c>
+      <c r="F98" t="s">
         <v>210</v>
       </c>
     </row>

</xml_diff>